<commit_message>
feat: separate cohort tracker + static HTML docs site
- Moved cohort tracker to facilitator/DQ_HOL_Cohort_Tracker.xlsx (20 students,
  auto-calculating completion %, NPS, cohort metrics)
- Removed Cohort Tracker sheet from student feedback form
- Generated docs/ static HTML site from markdown sources with:
  - Snowflake-branded CSS (blue headers, dark nav, alternating rows)
  - Mermaid.js for diagram rendering
  - Navigation bar across all pages
  - Offline-friendly (single HTML files, CDN for mermaid only)

.... Generated with [Cortex Code](https://docs.snowflake.com/en/user-guide/cortex-code/cortex-code)

Co-Authored-By: Cortex Code <noreply@snowflake.com>
</commit_message>
<xml_diff>
--- a/guide/DQ_HOL_Feedback_Form.xlsx
+++ b/guide/DQ_HOL_Feedback_Form.xlsx
@@ -9,7 +9,6 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module Feedback" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Enhancement Requests" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohort Tracker" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1288,553 +1287,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:P29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="5" customWidth="1" min="5" max="5"/>
-    <col width="5" customWidth="1" min="6" max="6"/>
-    <col width="5" customWidth="1" min="7" max="7"/>
-    <col width="5" customWidth="1" min="8" max="8"/>
-    <col width="5" customWidth="1" min="9" max="9"/>
-    <col width="5" customWidth="1" min="10" max="10"/>
-    <col width="5" customWidth="1" min="11" max="11"/>
-    <col width="6" customWidth="1" min="12" max="12"/>
-    <col width="5" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="6" customWidth="1" min="15" max="15"/>
-    <col width="30" customWidth="1" min="16" max="16"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Partner Cohort Progress Tracker</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Cohort Name:</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Partner:</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Start Date:</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Facilitator:</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Student Name</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Role</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>M0</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>M0B</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>M1</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>M2</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>M3</t>
-        </is>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>M4</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>M5</t>
-        </is>
-      </c>
-      <c r="L6" s="3" t="inlineStr">
-        <is>
-          <t>M6-7</t>
-        </is>
-      </c>
-      <c r="M6" s="3" t="inlineStr">
-        <is>
-          <t>M8</t>
-        </is>
-      </c>
-      <c r="N6" s="3" t="inlineStr">
-        <is>
-          <t>Completion %</t>
-        </is>
-      </c>
-      <c r="O6" s="3" t="inlineStr">
-        <is>
-          <t>NPS</t>
-        </is>
-      </c>
-      <c r="P6" s="3" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="n"/>
-      <c r="J7" s="5" t="n"/>
-      <c r="K7" s="5" t="n"/>
-      <c r="L7" s="5" t="n"/>
-      <c r="M7" s="5" t="n"/>
-      <c r="N7" s="5">
-        <f>COUNTIF(E7:M7,"Y")/9*100</f>
-        <v/>
-      </c>
-      <c r="O7" s="5" t="n"/>
-      <c r="P7" s="5" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="B8" s="4" t="n"/>
-      <c r="C8" s="4" t="n"/>
-      <c r="D8" s="4" t="n"/>
-      <c r="E8" s="4" t="n"/>
-      <c r="F8" s="4" t="n"/>
-      <c r="G8" s="4" t="n"/>
-      <c r="H8" s="4" t="n"/>
-      <c r="I8" s="4" t="n"/>
-      <c r="J8" s="4" t="n"/>
-      <c r="K8" s="4" t="n"/>
-      <c r="L8" s="4" t="n"/>
-      <c r="M8" s="4" t="n"/>
-      <c r="N8" s="4">
-        <f>COUNTIF(E8:M8,"Y")/9*100</f>
-        <v/>
-      </c>
-      <c r="O8" s="4" t="n"/>
-      <c r="P8" s="4" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="n"/>
-      <c r="J9" s="5" t="n"/>
-      <c r="K9" s="5" t="n"/>
-      <c r="L9" s="5" t="n"/>
-      <c r="M9" s="5" t="n"/>
-      <c r="N9" s="5">
-        <f>COUNTIF(E9:M9,"Y")/9*100</f>
-        <v/>
-      </c>
-      <c r="O9" s="5" t="n"/>
-      <c r="P9" s="5" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B10" s="4" t="n"/>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="4" t="n"/>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="4" t="n"/>
-      <c r="G10" s="4" t="n"/>
-      <c r="H10" s="4" t="n"/>
-      <c r="I10" s="4" t="n"/>
-      <c r="J10" s="4" t="n"/>
-      <c r="K10" s="4" t="n"/>
-      <c r="L10" s="4" t="n"/>
-      <c r="M10" s="4" t="n"/>
-      <c r="N10" s="4">
-        <f>COUNTIF(E10:M10,"Y")/9*100</f>
-        <v/>
-      </c>
-      <c r="O10" s="4" t="n"/>
-      <c r="P10" s="4" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="5" t="n"/>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
-      <c r="I11" s="5" t="n"/>
-      <c r="J11" s="5" t="n"/>
-      <c r="K11" s="5" t="n"/>
-      <c r="L11" s="5" t="n"/>
-      <c r="M11" s="5" t="n"/>
-      <c r="N11" s="5">
-        <f>COUNTIF(E11:M11,"Y")/9*100</f>
-        <v/>
-      </c>
-      <c r="O11" s="5" t="n"/>
-      <c r="P11" s="5" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B12" s="4" t="n"/>
-      <c r="C12" s="4" t="n"/>
-      <c r="D12" s="4" t="n"/>
-      <c r="E12" s="4" t="n"/>
-      <c r="F12" s="4" t="n"/>
-      <c r="G12" s="4" t="n"/>
-      <c r="H12" s="4" t="n"/>
-      <c r="I12" s="4" t="n"/>
-      <c r="J12" s="4" t="n"/>
-      <c r="K12" s="4" t="n"/>
-      <c r="L12" s="4" t="n"/>
-      <c r="M12" s="4" t="n"/>
-      <c r="N12" s="4">
-        <f>COUNTIF(E12:M12,"Y")/9*100</f>
-        <v/>
-      </c>
-      <c r="O12" s="4" t="n"/>
-      <c r="P12" s="4" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="B13" s="5" t="n"/>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="5" t="n"/>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="n"/>
-      <c r="G13" s="5" t="n"/>
-      <c r="H13" s="5" t="n"/>
-      <c r="I13" s="5" t="n"/>
-      <c r="J13" s="5" t="n"/>
-      <c r="K13" s="5" t="n"/>
-      <c r="L13" s="5" t="n"/>
-      <c r="M13" s="5" t="n"/>
-      <c r="N13" s="5">
-        <f>COUNTIF(E13:M13,"Y")/9*100</f>
-        <v/>
-      </c>
-      <c r="O13" s="5" t="n"/>
-      <c r="P13" s="5" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="B14" s="4" t="n"/>
-      <c r="C14" s="4" t="n"/>
-      <c r="D14" s="4" t="n"/>
-      <c r="E14" s="4" t="n"/>
-      <c r="F14" s="4" t="n"/>
-      <c r="G14" s="4" t="n"/>
-      <c r="H14" s="4" t="n"/>
-      <c r="I14" s="4" t="n"/>
-      <c r="J14" s="4" t="n"/>
-      <c r="K14" s="4" t="n"/>
-      <c r="L14" s="4" t="n"/>
-      <c r="M14" s="4" t="n"/>
-      <c r="N14" s="4">
-        <f>COUNTIF(E14:M14,"Y")/9*100</f>
-        <v/>
-      </c>
-      <c r="O14" s="4" t="n"/>
-      <c r="P14" s="4" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="5" t="n"/>
-      <c r="D15" s="5" t="n"/>
-      <c r="E15" s="5" t="n"/>
-      <c r="F15" s="5" t="n"/>
-      <c r="G15" s="5" t="n"/>
-      <c r="H15" s="5" t="n"/>
-      <c r="I15" s="5" t="n"/>
-      <c r="J15" s="5" t="n"/>
-      <c r="K15" s="5" t="n"/>
-      <c r="L15" s="5" t="n"/>
-      <c r="M15" s="5" t="n"/>
-      <c r="N15" s="5">
-        <f>COUNTIF(E15:M15,"Y")/9*100</f>
-        <v/>
-      </c>
-      <c r="O15" s="5" t="n"/>
-      <c r="P15" s="5" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="B16" s="4" t="n"/>
-      <c r="C16" s="4" t="n"/>
-      <c r="D16" s="4" t="n"/>
-      <c r="E16" s="4" t="n"/>
-      <c r="F16" s="4" t="n"/>
-      <c r="G16" s="4" t="n"/>
-      <c r="H16" s="4" t="n"/>
-      <c r="I16" s="4" t="n"/>
-      <c r="J16" s="4" t="n"/>
-      <c r="K16" s="4" t="n"/>
-      <c r="L16" s="4" t="n"/>
-      <c r="M16" s="4" t="n"/>
-      <c r="N16" s="4">
-        <f>COUNTIF(E16:M16,"Y")/9*100</f>
-        <v/>
-      </c>
-      <c r="O16" s="4" t="n"/>
-      <c r="P16" s="4" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="n">
-        <v>11</v>
-      </c>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="5" t="n"/>
-      <c r="E17" s="5" t="n"/>
-      <c r="F17" s="5" t="n"/>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="n"/>
-      <c r="I17" s="5" t="n"/>
-      <c r="J17" s="5" t="n"/>
-      <c r="K17" s="5" t="n"/>
-      <c r="L17" s="5" t="n"/>
-      <c r="M17" s="5" t="n"/>
-      <c r="N17" s="5">
-        <f>COUNTIF(E17:M17,"Y")/9*100</f>
-        <v/>
-      </c>
-      <c r="O17" s="5" t="n"/>
-      <c r="P17" s="5" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="B18" s="4" t="n"/>
-      <c r="C18" s="4" t="n"/>
-      <c r="D18" s="4" t="n"/>
-      <c r="E18" s="4" t="n"/>
-      <c r="F18" s="4" t="n"/>
-      <c r="G18" s="4" t="n"/>
-      <c r="H18" s="4" t="n"/>
-      <c r="I18" s="4" t="n"/>
-      <c r="J18" s="4" t="n"/>
-      <c r="K18" s="4" t="n"/>
-      <c r="L18" s="4" t="n"/>
-      <c r="M18" s="4" t="n"/>
-      <c r="N18" s="4">
-        <f>COUNTIF(E18:M18,"Y")/9*100</f>
-        <v/>
-      </c>
-      <c r="O18" s="4" t="n"/>
-      <c r="P18" s="4" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="B19" s="5" t="n"/>
-      <c r="C19" s="5" t="n"/>
-      <c r="D19" s="5" t="n"/>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="5" t="n"/>
-      <c r="G19" s="5" t="n"/>
-      <c r="H19" s="5" t="n"/>
-      <c r="I19" s="5" t="n"/>
-      <c r="J19" s="5" t="n"/>
-      <c r="K19" s="5" t="n"/>
-      <c r="L19" s="5" t="n"/>
-      <c r="M19" s="5" t="n"/>
-      <c r="N19" s="5">
-        <f>COUNTIF(E19:M19,"Y")/9*100</f>
-        <v/>
-      </c>
-      <c r="O19" s="5" t="n"/>
-      <c r="P19" s="5" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="B20" s="4" t="n"/>
-      <c r="C20" s="4" t="n"/>
-      <c r="D20" s="4" t="n"/>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="4" t="n"/>
-      <c r="G20" s="4" t="n"/>
-      <c r="H20" s="4" t="n"/>
-      <c r="I20" s="4" t="n"/>
-      <c r="J20" s="4" t="n"/>
-      <c r="K20" s="4" t="n"/>
-      <c r="L20" s="4" t="n"/>
-      <c r="M20" s="4" t="n"/>
-      <c r="N20" s="4">
-        <f>COUNTIF(E20:M20,"Y")/9*100</f>
-        <v/>
-      </c>
-      <c r="O20" s="4" t="n"/>
-      <c r="P20" s="4" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="B21" s="5" t="n"/>
-      <c r="C21" s="5" t="n"/>
-      <c r="D21" s="5" t="n"/>
-      <c r="E21" s="5" t="n"/>
-      <c r="F21" s="5" t="n"/>
-      <c r="G21" s="5" t="n"/>
-      <c r="H21" s="5" t="n"/>
-      <c r="I21" s="5" t="n"/>
-      <c r="J21" s="5" t="n"/>
-      <c r="K21" s="5" t="n"/>
-      <c r="L21" s="5" t="n"/>
-      <c r="M21" s="5" t="n"/>
-      <c r="N21" s="5">
-        <f>COUNTIF(E21:M21,"Y")/9*100</f>
-        <v/>
-      </c>
-      <c r="O21" s="5" t="n"/>
-      <c r="P21" s="5" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>COHORT SUMMARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t>Total Students:</t>
-        </is>
-      </c>
-      <c r="B24" s="6">
-        <f>COUNTA(B7:B21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t>Avg Completion %:</t>
-        </is>
-      </c>
-      <c r="B25" s="6">
-        <f>AVERAGE(N7:N21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>Avg NPS:</t>
-        </is>
-      </c>
-      <c r="B26" s="6">
-        <f>AVERAGE(O7:O21)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>Full Completion Rate:</t>
-        </is>
-      </c>
-      <c r="B27" s="6">
-        <f>COUNTIF(N7:N21,"&gt;=100")/COUNTA(B7:B21)*100</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="8" t="inlineStr">
-        <is>
-          <t>Mark Y in module columns when student completes. Completion % auto-calculates.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:N1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>